<commit_message>
restore module READMEs; ATLAS tactic rename; recalc M03 starter
</commit_message>
<xml_diff>
--- a/03_ai-threat-modeling-mitre-atlas/demo/threat_model_demo.xlsx
+++ b/03_ai-threat-modeling-mitre-atlas/demo/threat_model_demo.xlsx
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>ML Attack Staging</t>
+          <t>AI Attack Staging</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="B3" s="22" t="inlineStr">
         <is>
-          <t>ATLAS lists Backdoor AI Model under both "Persistence" and "ML Attack Staging" tactics, depending on whether the backdoor is staged before deployment or seeded post-deployment.</t>
+          <t>ATLAS lists Backdoor AI Model under both "Persistence" and "AI Attack Staging" tactics, depending on whether the backdoor is staged before deployment or seeded post-deployment.</t>
         </is>
       </c>
     </row>

</xml_diff>